<commit_message>
Use optional column "expressed_as" for aquatic toxicity
Also, Marcel added boscalid fish toxicity from the RAR LoEP, and
changed the representation of the data for naphthylacetic acid
when tested as the sodium salt. Now the sodium salt is given
as "formulation", similar to the way we are showing data for copper
compounds, where the copper compounds are listed as "formulation" as
well, although strictly speaking they are not formulations.
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/1-naphthylacetic_acid_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/1-naphthylacetic_acid_aquatic_toxicity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16649F92-B193-4C6E-911A-C1FC7348AD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EB04FC5-58FA-416D-B6B0-3B61FD6F879C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aquatic_endpoints" sheetId="6" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="64">
   <si>
     <t>Oncorhynchus mykiss</t>
   </si>
@@ -220,15 +220,6 @@
   </si>
   <si>
     <t>1-Naphthylacetic acid sodium salt</t>
-  </si>
-  <si>
-    <t>Reported as &gt;82 mg/L 1-naphthylacetic acid</t>
-  </si>
-  <si>
-    <t>Reported as 18,05 mg/L 1-naphthylacetic acid</t>
-  </si>
-  <si>
-    <t>Reported as 26,62 mg/L 1-naphthylacetic acid</t>
   </si>
   <si>
     <t>TRUE</t>
@@ -287,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -304,6 +295,9 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -587,32 +581,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C316ADCA-0F97-4E34-A600-B1604EAF90B0}">
   <dimension ref="A1:X24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" style="3" customWidth="1"/>
-    <col min="2" max="2" width="16.54296875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="7.453125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="13.1796875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="22.453125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="9.453125" style="3"/>
-    <col min="9" max="9" width="9.453125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="14.26953125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="9.453125" style="3"/>
-    <col min="12" max="12" width="5.54296875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="12.7265625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" style="3"/>
-    <col min="15" max="15" width="11.7265625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="17.453125" style="3" customWidth="1"/>
-    <col min="17" max="17" width="9.453125" style="3"/>
-    <col min="18" max="18" width="14.26953125" style="3" customWidth="1"/>
-    <col min="19" max="19" width="13.1796875" style="3" customWidth="1"/>
-    <col min="20" max="20" width="9.453125" style="4"/>
-    <col min="21" max="16384" width="9.453125" style="3"/>
+    <col min="2" max="2" width="16.5703125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="7.42578125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="22.42578125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="8.5703125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" style="3"/>
+    <col min="9" max="9" width="9.42578125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" style="3"/>
+    <col min="12" max="12" width="5.5703125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" style="3"/>
+    <col min="15" max="15" width="11.7109375" style="3" customWidth="1"/>
+    <col min="16" max="16" width="17.42578125" style="3" customWidth="1"/>
+    <col min="17" max="17" width="9.42578125" style="3"/>
+    <col min="18" max="18" width="14.28515625" style="3" customWidth="1"/>
+    <col min="19" max="19" width="13.140625" style="3" customWidth="1"/>
+    <col min="20" max="20" width="9.42578125" style="4"/>
+    <col min="21" max="16384" width="9.42578125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>21</v>
       </c>
@@ -686,7 +680,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>59</v>
       </c>
@@ -733,10 +727,10 @@
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
       <c r="T2" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U2" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V2" s="7"/>
       <c r="W2" s="5" t="s">
@@ -746,7 +740,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>59</v>
       </c>
@@ -791,10 +785,10 @@
         <v>43</v>
       </c>
       <c r="T3" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V3" s="7"/>
       <c r="W3" s="5" t="s">
@@ -804,11 +798,13 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="7"/>
       <c r="C4" s="7" t="s">
         <v>44</v>
       </c>
@@ -831,8 +827,7 @@
         <v>34</v>
       </c>
       <c r="M4" s="6">
-        <f>82*(208.19/186.21)</f>
-        <v>91.679179421083731</v>
+        <v>82</v>
       </c>
       <c r="N4" s="7" t="s">
         <v>14</v>
@@ -847,22 +842,20 @@
         <v>43</v>
       </c>
       <c r="T4" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U4" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="V4" s="7" t="s">
-        <v>61</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="V4" s="7"/>
       <c r="W4" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="X4" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="X4" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>59</v>
       </c>
@@ -905,10 +898,10 @@
         <v>43</v>
       </c>
       <c r="T5" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U5" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V5" s="7"/>
       <c r="W5" s="5" t="s">
@@ -918,7 +911,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>59</v>
       </c>
@@ -963,10 +956,10 @@
         <v>43</v>
       </c>
       <c r="T6" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U6" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V6" s="7"/>
       <c r="W6" s="5" t="s">
@@ -976,7 +969,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>59</v>
       </c>
@@ -1019,10 +1012,10 @@
         <v>43</v>
       </c>
       <c r="T7" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U7" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V7" s="7"/>
       <c r="W7" s="5" t="s">
@@ -1032,7 +1025,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>59</v>
       </c>
@@ -1077,10 +1070,10 @@
         <v>43</v>
       </c>
       <c r="T8" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U8" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V8" s="7"/>
       <c r="W8" s="5" t="s">
@@ -1090,7 +1083,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>59</v>
       </c>
@@ -1135,10 +1128,10 @@
         <v>43</v>
       </c>
       <c r="T9" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U9" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V9" s="7"/>
       <c r="W9" s="5" t="s">
@@ -1148,11 +1141,13 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="7"/>
       <c r="C10" s="7" t="s">
         <v>1</v>
       </c>
@@ -1175,8 +1170,7 @@
         <v>34</v>
       </c>
       <c r="M10" s="6">
-        <f>82*(208.19/186.21)</f>
-        <v>91.679179421083731</v>
+        <v>82</v>
       </c>
       <c r="N10" s="7" t="s">
         <v>14</v>
@@ -1191,22 +1185,20 @@
         <v>43</v>
       </c>
       <c r="T10" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U10" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="V10" s="7" t="s">
-        <v>61</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="V10" s="7"/>
       <c r="W10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="X10" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+      <c r="X10" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>59</v>
       </c>
@@ -1249,10 +1241,10 @@
         <v>43</v>
       </c>
       <c r="T11" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U11" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V11" s="7"/>
       <c r="W11" s="5" t="s">
@@ -1262,7 +1254,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:24" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>59</v>
       </c>
@@ -1309,10 +1301,10 @@
         <v>43</v>
       </c>
       <c r="T12" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U12" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V12" s="7" t="s">
         <v>56</v>
@@ -1324,7 +1316,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>59</v>
       </c>
@@ -1367,10 +1359,10 @@
         <v>43</v>
       </c>
       <c r="T13" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U13" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V13" s="7"/>
       <c r="W13" s="5" t="s">
@@ -1380,7 +1372,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>59</v>
       </c>
@@ -1425,10 +1417,10 @@
         <v>43</v>
       </c>
       <c r="T14" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U14" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V14" s="7"/>
       <c r="W14" s="5" t="s">
@@ -1438,7 +1430,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>59</v>
       </c>
@@ -1479,10 +1471,10 @@
         <v>43</v>
       </c>
       <c r="T15" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U15" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V15" s="7"/>
       <c r="W15" s="5" t="s">
@@ -1492,7 +1484,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>59</v>
       </c>
@@ -1533,10 +1525,10 @@
         <v>43</v>
       </c>
       <c r="T16" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U16" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V16" s="7"/>
       <c r="W16" s="5" t="s">
@@ -1546,11 +1538,13 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="7"/>
       <c r="C17" s="7" t="s">
         <v>40</v>
       </c>
@@ -1574,8 +1568,7 @@
       </c>
       <c r="L17" s="7"/>
       <c r="M17" s="6">
-        <f>18.05*(208.19/186.21)</f>
-        <v>20.180599860372698</v>
+        <v>18.05</v>
       </c>
       <c r="N17" s="7" t="s">
         <v>14</v>
@@ -1590,26 +1583,26 @@
         <v>43</v>
       </c>
       <c r="T17" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U17" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="V17" s="7" t="s">
-        <v>62</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="V17" s="7"/>
       <c r="W17" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="X17" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="18" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="X17" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="7"/>
       <c r="C18" s="7" t="s">
         <v>40</v>
       </c>
@@ -1633,8 +1626,7 @@
       </c>
       <c r="L18" s="7"/>
       <c r="M18" s="6">
-        <f>26.62*(208.19/186.21)</f>
-        <v>29.762192148649376</v>
+        <v>26.62</v>
       </c>
       <c r="N18" s="7" t="s">
         <v>14</v>
@@ -1649,22 +1641,20 @@
         <v>43</v>
       </c>
       <c r="T18" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U18" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="V18" s="7" t="s">
-        <v>63</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="V18" s="7"/>
       <c r="W18" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="X18" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="X18" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>59</v>
       </c>
@@ -1709,10 +1699,10 @@
         <v>43</v>
       </c>
       <c r="T19" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U19" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V19" s="7" t="s">
         <v>56</v>
@@ -1724,7 +1714,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:24" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>59</v>
       </c>
@@ -1771,10 +1761,10 @@
         <v>43</v>
       </c>
       <c r="T20" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U20" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V20" s="7" t="s">
         <v>56</v>
@@ -1786,7 +1776,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>59</v>
       </c>
@@ -1831,10 +1821,10 @@
         <v>43</v>
       </c>
       <c r="T21" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U21" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V21" s="7"/>
       <c r="W21" s="5" t="s">
@@ -1844,7 +1834,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>59</v>
       </c>
@@ -1889,10 +1879,10 @@
         <v>43</v>
       </c>
       <c r="T22" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U22" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V22" s="7"/>
       <c r="W22" s="5" t="s">
@@ -1902,7 +1892,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>59</v>
       </c>
@@ -1910,7 +1900,7 @@
         <v>50</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D23" s="6">
         <v>16</v>
@@ -1949,10 +1939,10 @@
         <v>43</v>
       </c>
       <c r="T23" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U23" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V23" s="7"/>
       <c r="W23" s="5" t="s">
@@ -1962,7 +1952,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:24" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>59</v>
       </c>
@@ -1970,7 +1960,7 @@
         <v>53</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D24" s="6">
         <v>17</v>
@@ -2009,10 +1999,10 @@
         <v>43</v>
       </c>
       <c r="T24" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="U24" s="7" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="V24" s="7"/>
       <c r="W24" s="5" t="s">

</xml_diff>